<commit_message>
Update pipeline, results, and plots
</commit_message>
<xml_diff>
--- a/outputs/model_results.xlsx
+++ b/outputs/model_results.xlsx
@@ -12,7 +12,7 @@
     <sheet name="gbr_cv_results" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="gbr_built_in_feature_importance" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="gbr_permutation_importance" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="gbr_shap_importance_error" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="gbr_shap_importance" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="hgbr_metrics" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="hgbr_cv_results" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="hgbr_permutation_importance" sheetId="9" state="visible" r:id="rId9"/>
@@ -457,19 +457,19 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.4534769571401892</v>
+        <v>0.4793444018779683</v>
       </c>
       <c r="B2" t="n">
-        <v>2.07562473934563</v>
+        <v>2.274137744998793</v>
       </c>
       <c r="C2" t="n">
-        <v>6.925124234820434</v>
+        <v>8.437571960529963</v>
       </c>
       <c r="D2" t="n">
-        <v>2.631563078252245</v>
+        <v>2.90474989638178</v>
       </c>
       <c r="E2" t="n">
-        <v>0.4756038570432534</v>
+        <v>0.4029318613521077</v>
       </c>
     </row>
   </sheetData>
@@ -505,17 +505,17 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8174403695652436</v>
+        <v>0.702169412282209</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>categoricals__bitsize_24</t>
+          <t>numericals__flowrate</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.709106984438712</v>
+        <v>0.701103922807134</v>
       </c>
     </row>
     <row r="4">
@@ -525,17 +525,17 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.6429734446616171</v>
+        <v>0.6327719242547558</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>numericals__flowrate</t>
+          <t>categoricals__bitsize_24</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.5526711354232005</v>
+        <v>0.597947519280164</v>
       </c>
     </row>
     <row r="6">
@@ -545,67 +545,67 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.4316115155418565</v>
+        <v>0.2804249978699422</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>numericals__rpm</t>
+          <t>numericals__spp</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.3643992597035506</v>
+        <v>0.2383160958549066</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>numericals__spp</t>
+          <t>numericals__rpm</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.3071444409915065</v>
+        <v>0.1716623881666661</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>categoricals__bitsize_17</t>
+          <t>categoricals__bitsize_8.5</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.2631281757709929</v>
+        <v>0.05255826080307155</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>categoricals__bitsize_8.5</t>
+          <t>categoricals__bitsize_17</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.1540682138403352</v>
+        <v>0.04446272426082877</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>categoricals__bitsize_12</t>
+          <t>categoricals__bitsize_26</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.06611191038142895</v>
+        <v>0.002756471233089202</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>categoricals__bitsize_26</t>
+          <t>categoricals__bitsize_12</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.03455788319471724</v>
+        <v>0.001257251484506512</v>
       </c>
     </row>
     <row r="13">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.004625527524216952</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -661,19 +661,19 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.811931557979099</v>
+        <v>0.8389802439375325</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7973017894213033</v>
+        <v>0.638747890207024</v>
       </c>
       <c r="C2" t="n">
-        <v>1.105908759563835</v>
+        <v>1.601796747689544</v>
       </c>
       <c r="D2" t="n">
-        <v>2.676812767002082</v>
+        <v>5.105096847361756</v>
       </c>
       <c r="E2" t="n">
-        <v>1.636096808566682</v>
+        <v>2.259446137300413</v>
       </c>
     </row>
   </sheetData>
@@ -724,22 +724,22 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1.027514457702637</v>
+        <v>1.621323347091675</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8435707092285156</v>
+        <v>0.627777099609375</v>
       </c>
       <c r="C2" t="n">
-        <v>1.075701117515564</v>
+        <v>1.98991322517395</v>
       </c>
       <c r="D2" t="n">
-        <v>2.286297798156738</v>
+        <v>6.897231578826904</v>
       </c>
       <c r="E2" t="n">
-        <v>1.512050858323469</v>
+        <v>2.626258094480987</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8268730640411377</v>
+        <v>0.5119310021400452</v>
       </c>
     </row>
   </sheetData>
@@ -850,19 +850,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.4534769571401892</v>
+        <v>0.4793444018779683</v>
       </c>
       <c r="D2" t="n">
-        <v>2.07562473934563</v>
+        <v>2.274137744998793</v>
       </c>
       <c r="E2" t="n">
-        <v>6.925124234820434</v>
+        <v>8.437571960529963</v>
       </c>
       <c r="F2" t="n">
-        <v>2.631563078252245</v>
+        <v>2.90474989638178</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4756038570432534</v>
+        <v>0.4029318613521077</v>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
@@ -886,27 +886,27 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.737189473933591</v>
+        <v>0.5438284837349614</v>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>0.7358894906408787</v>
+        <v>0.4538846253503861</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__learning_rate': 0.061679538755918244, 'model__loss': 'huber', 'model__max_depth': 3, 'model__max_features': 'log2', 'model__min_samples_leaf': 13, 'model__min_samples_split': 13, 'model__n_estimators': 148, 'model__n_iter_no_change': 14, 'model__subsample': 0.8279822153767209, 'model__tol': 5.937320984080647e-05, 'model__validation_fraction': 0.13415957421026364})</t>
+          <t>OrderedDict({'model__learning_rate': 0.03705491779715134, 'model__loss': 'absolute_error', 'model__max_depth': 2, 'model__max_features': 'sqrt', 'model__min_samples_leaf': 8, 'model__min_samples_split': 24, 'model__n_estimators': 70, 'model__n_iter_no_change': 13, 'model__subsample': 0.7393351057584503, 'model__tol': 0.0008839220247589657, 'model__validation_fraction': 0.1703467531106304})</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>1.352894015848332</v>
+        <v>2.101408004237677</v>
       </c>
       <c r="J3" t="n">
-        <v>1.867569967962211</v>
+        <v>2.778043221140134</v>
       </c>
       <c r="K3" t="n">
-        <v>0.001299983292712303</v>
+        <v>0.0899438583845753</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
@@ -926,39 +926,39 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.8688782618292484</v>
+        <v>0.6750586454318424</v>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>0.8435790319421856</v>
+        <v>0.5448982864179632</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__l2_regularization': 1.0889237550644373, 'model__learning_rate': 0.0696604761871229, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 596, 'model__max_leaf_nodes': 22, 'model__min_samples_leaf': 59, 'model__n_iter_no_change': 18, 'model__tol': 0.00029360602985208155, 'model__validation_fraction': 0.20245894424862895})</t>
+          <t>OrderedDict({'model__l2_regularization': 1.3143839143527278, 'model__learning_rate': 0.020000000000000004, 'model__loss': 'squared_error', 'model__max_depth': 2, 'model__max_iter': 300, 'model__max_leaf_nodes': 31, 'model__min_samples_leaf': 80, 'model__n_iter_no_change': 10, 'model__tol': 6.185326471010234e-05, 'model__validation_fraction': 0.25})</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>1.04025269998195</v>
+        <v>1.957518884701225</v>
       </c>
       <c r="J4" t="n">
-        <v>1.437247377164544</v>
+        <v>2.53601041030362</v>
       </c>
       <c r="K4" t="n">
-        <v>0.02529922988706279</v>
+        <v>0.1301603590138791</v>
       </c>
       <c r="L4" t="n">
-        <v>0.8635426478146394</v>
+        <v>0.7588469253790955</v>
       </c>
       <c r="M4" t="n">
-        <v>0.7876187444750997</v>
+        <v>-0.07476905660647337</v>
       </c>
       <c r="N4" t="n">
-        <v>0.07592390333953969</v>
+        <v>0.8336159819855689</v>
       </c>
       <c r="O4" t="n">
-        <v>0.7496567928053299</v>
+        <v>-0.4915770475992578</v>
       </c>
       <c r="P4" t="inlineStr"/>
     </row>
@@ -974,19 +974,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.811931557979099</v>
+        <v>0.8389802439375325</v>
       </c>
       <c r="D5" t="n">
-        <v>1.105908759563835</v>
+        <v>1.601796747689544</v>
       </c>
       <c r="E5" t="n">
-        <v>2.676812767002082</v>
+        <v>5.105096847361756</v>
       </c>
       <c r="F5" t="n">
-        <v>1.636096808566682</v>
+        <v>2.259446137300413</v>
       </c>
       <c r="G5" t="n">
-        <v>0.7973017894213033</v>
+        <v>0.638747890207024</v>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
@@ -1010,19 +1010,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.8435707092285156</v>
+        <v>0.627777099609375</v>
       </c>
       <c r="D6" t="n">
-        <v>1.075701117515564</v>
+        <v>1.98991322517395</v>
       </c>
       <c r="E6" t="n">
-        <v>2.286297798156738</v>
+        <v>6.897231578826904</v>
       </c>
       <c r="F6" t="n">
-        <v>1.512050858323469</v>
+        <v>2.626258094480987</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8268730640411377</v>
+        <v>0.5119310021400452</v>
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
@@ -1033,7 +1033,7 @@
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="n">
-        <v>1.027514457702637</v>
+        <v>1.621323347091675</v>
       </c>
     </row>
   </sheetData>
@@ -1085,23 +1085,23 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__learning_rate': 0.061679538755918244, 'model__loss': 'huber', 'model__max_depth': 3, 'model__max_features': 'log2', 'model__min_samples_leaf': 13, 'model__min_samples_split': 13, 'model__n_estimators': 148, 'model__n_iter_no_change': 14, 'model__subsample': 0.8279822153767209, 'model__tol': 5.937320984080647e-05, 'model__validation_fraction': 0.13415957421026364})</t>
+          <t>OrderedDict({'model__learning_rate': 0.03705491779715134, 'model__loss': 'absolute_error', 'model__max_depth': 2, 'model__max_features': 'sqrt', 'model__min_samples_leaf': 8, 'model__min_samples_split': 24, 'model__n_estimators': 70, 'model__n_iter_no_change': 13, 'model__subsample': 0.7393351057584503, 'model__tol': 0.0008839220247589657, 'model__validation_fraction': 0.1703467531106304})</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.737189473933591</v>
+        <v>0.5438284837349614</v>
       </c>
       <c r="C2" t="n">
-        <v>0.7358894906408787</v>
+        <v>0.4538846253503861</v>
       </c>
       <c r="D2" t="n">
-        <v>1.352894015848332</v>
+        <v>2.101408004237677</v>
       </c>
       <c r="E2" t="n">
-        <v>1.867569967962211</v>
+        <v>2.778043221140134</v>
       </c>
       <c r="F2" t="n">
-        <v>0.001299983292712303</v>
+        <v>0.0899438583845753</v>
       </c>
     </row>
   </sheetData>
@@ -1252,113 +1252,113 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.4033478498458862</v>
+        <v>0.1711235046386719</v>
       </c>
       <c r="B2" t="n">
-        <v>0.001500964164733887</v>
+        <v>0.0002465248107910156</v>
       </c>
       <c r="C2" t="n">
-        <v>0.007359981536865234</v>
+        <v>0.006762146949768066</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0003483295440673828</v>
+        <v>0.0002471208572387695</v>
       </c>
       <c r="E2" t="n">
-        <v>0.06167953875591824</v>
+        <v>0.03705491779715134</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>huber</t>
+          <t>absolute_error</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>log2</t>
+          <t>sqrt</t>
         </is>
       </c>
       <c r="I2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J2" t="n">
+        <v>24</v>
+      </c>
+      <c r="K2" t="n">
+        <v>70</v>
+      </c>
+      <c r="L2" t="n">
         <v>13</v>
       </c>
-      <c r="J2" t="n">
-        <v>13</v>
-      </c>
-      <c r="K2" t="n">
-        <v>148</v>
-      </c>
-      <c r="L2" t="n">
-        <v>14</v>
-      </c>
       <c r="M2" t="n">
-        <v>0.8279822153767209</v>
+        <v>0.7393351057584503</v>
       </c>
       <c r="N2" t="n">
-        <v>5.937320984080647e-05</v>
+        <v>0.0008839220247589657</v>
       </c>
       <c r="O2" t="n">
-        <v>0.1341595742102636</v>
+        <v>0.1703467531106304</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__learning_rate': 0.061679538755918244, 'model__loss': 'huber', 'model__max_depth': 3, 'model__max_features': 'log2', 'model__min_samples_leaf': 13, 'model__min_samples_split': 13, 'model__n_estimators': 148, 'model__n_iter_no_change': 14, 'model__subsample': 0.8279822153767209, 'model__tol': 5.937320984080647e-05, 'model__validation_fraction': 0.13415957421026364})</t>
+          <t>OrderedDict({'model__learning_rate': 0.03705491779715134, 'model__loss': 'absolute_error', 'model__max_depth': 2, 'model__max_features': 'sqrt', 'model__min_samples_leaf': 8, 'model__min_samples_split': 24, 'model__n_estimators': 70, 'model__n_iter_no_change': 13, 'model__subsample': 0.7393351057584503, 'model__tol': 0.0008839220247589657, 'model__validation_fraction': 0.1703467531106304})</t>
         </is>
       </c>
       <c r="Q2" t="n">
-        <v>0.7014956889982324</v>
+        <v>-0.0424503644320311</v>
       </c>
       <c r="R2" t="n">
-        <v>0.7295541267146246</v>
+        <v>0.0567423398157415</v>
       </c>
       <c r="S2" t="n">
-        <v>0.7155249078564285</v>
+        <v>0.007145987691855205</v>
       </c>
       <c r="T2" t="n">
-        <v>0.01402921885819608</v>
+        <v>0.0495963521238863</v>
       </c>
       <c r="U2" t="n">
         <v>1</v>
       </c>
       <c r="V2" t="n">
-        <v>0.7546729552498612</v>
+        <v>0.5786914165540138</v>
       </c>
       <c r="W2" t="n">
-        <v>0.7405131015252093</v>
+        <v>0.6992520129182331</v>
       </c>
       <c r="X2" t="n">
-        <v>0.7475930283875353</v>
+        <v>0.6389717147361235</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.007079926862325947</v>
+        <v>0.06028029818210967</v>
       </c>
       <c r="Z2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.3240915536880493</v>
+        <v>0.1386218070983887</v>
       </c>
       <c r="B3" t="n">
-        <v>0.003490567207336426</v>
+        <v>0.0009894371032714844</v>
       </c>
       <c r="C3" t="n">
-        <v>0.006849527359008789</v>
+        <v>0.005760788917541504</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0008666515350341797</v>
+        <v>0.0002411603927612305</v>
       </c>
       <c r="E3" t="n">
-        <v>0.06059114141190369</v>
+        <v>0.06385398733009987</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>huber</t>
+          <t>absolute_error</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -1366,74 +1366,74 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J3" t="n">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="K3" t="n">
-        <v>105</v>
+        <v>68</v>
       </c>
       <c r="L3" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="M3" t="n">
-        <v>0.6882709613819928</v>
+        <v>0.7589322754697926</v>
       </c>
       <c r="N3" t="n">
-        <v>0.0002083782840547887</v>
+        <v>0.0008071612428512736</v>
       </c>
       <c r="O3" t="n">
-        <v>0.1512987949491055</v>
+        <v>0.162990106648119</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__learning_rate': 0.060591141411903686, 'model__loss': 'huber', 'model__max_depth': 3, 'model__max_features': 'log2', 'model__min_samples_leaf': 19, 'model__min_samples_split': 32, 'model__n_estimators': 105, 'model__n_iter_no_change': 12, 'model__subsample': 0.6882709613819928, 'model__tol': 0.00020837828405478867, 'model__validation_fraction': 0.15129879494910548})</t>
+          <t>OrderedDict({'model__learning_rate': 0.06385398733009987, 'model__loss': 'absolute_error', 'model__max_depth': 2, 'model__max_features': 'log2', 'model__min_samples_leaf': 18, 'model__min_samples_split': 12, 'model__n_estimators': 68, 'model__n_iter_no_change': 9, 'model__subsample': 0.7589322754697926, 'model__tol': 0.0008071612428512736, 'model__validation_fraction': 0.16299010664811903})</t>
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>0.6673930245059015</v>
+        <v>-0.03913327715826798</v>
       </c>
       <c r="R3" t="n">
-        <v>0.7003328337489471</v>
+        <v>-0.01209784188811547</v>
       </c>
       <c r="S3" t="n">
-        <v>0.6838629291274243</v>
+        <v>-0.02561555952319172</v>
       </c>
       <c r="T3" t="n">
-        <v>0.01646990462152276</v>
+        <v>0.01351771763507625</v>
       </c>
       <c r="U3" t="n">
         <v>2</v>
       </c>
       <c r="V3" t="n">
-        <v>0.7217239224797167</v>
+        <v>0.6751175525451727</v>
       </c>
       <c r="W3" t="n">
-        <v>0.7003455671002821</v>
+        <v>0.7575153538311444</v>
       </c>
       <c r="X3" t="n">
-        <v>0.7110347447899994</v>
+        <v>0.7163164531881585</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.01068917768971733</v>
+        <v>0.04119890064298587</v>
       </c>
       <c r="Z3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.2201895713806152</v>
+        <v>0.2463139295578003</v>
       </c>
       <c r="B4" t="n">
-        <v>0.00030517578125</v>
+        <v>0.002541661262512207</v>
       </c>
       <c r="C4" t="n">
-        <v>0.006643176078796387</v>
+        <v>0.007008671760559082</v>
       </c>
       <c r="D4" t="n">
-        <v>3.850460052490234e-05</v>
+        <v>0.0005031824111938477</v>
       </c>
       <c r="E4" t="n">
         <v>0.03531320873882618</v>
@@ -1478,31 +1478,31 @@
         </is>
       </c>
       <c r="Q4" t="n">
-        <v>0.5845840967012821</v>
+        <v>-0.0375206739242937</v>
       </c>
       <c r="R4" t="n">
-        <v>0.6242701117210694</v>
+        <v>-0.08010953699108736</v>
       </c>
       <c r="S4" t="n">
-        <v>0.6044271042111757</v>
+        <v>-0.05881510545769053</v>
       </c>
       <c r="T4" t="n">
-        <v>0.01984300750989365</v>
+        <v>0.02129443153339683</v>
       </c>
       <c r="U4" t="n">
         <v>3</v>
       </c>
       <c r="V4" t="n">
-        <v>0.6332050135422368</v>
+        <v>0.7344464438961724</v>
       </c>
       <c r="W4" t="n">
-        <v>0.6067813779787097</v>
+        <v>0.7964180057812998</v>
       </c>
       <c r="X4" t="n">
-        <v>0.6199931957604732</v>
+        <v>0.7654322248387362</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.01321181778176356</v>
+        <v>0.03098578094256371</v>
       </c>
       <c r="Z4" t="n">
         <v>3</v>
@@ -1510,27 +1510,27 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.1215415000915527</v>
+        <v>0.5501905679702759</v>
       </c>
       <c r="B5" t="n">
-        <v>0.001003265380859375</v>
+        <v>0.007264256477355957</v>
       </c>
       <c r="C5" t="n">
-        <v>0.005169391632080078</v>
+        <v>0.01051855087280273</v>
       </c>
       <c r="D5" t="n">
-        <v>0.001252889633178711</v>
+        <v>1.192092895507812e-06</v>
       </c>
       <c r="E5" t="n">
-        <v>0.06385398733009987</v>
+        <v>0.06167953875591824</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>absolute_error</t>
+          <t>huber</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1538,146 +1538,146 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="J5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K5" t="n">
-        <v>68</v>
+        <v>148</v>
       </c>
       <c r="L5" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="M5" t="n">
-        <v>0.7589322754697926</v>
+        <v>0.8279822153767209</v>
       </c>
       <c r="N5" t="n">
-        <v>0.0008071612428512736</v>
+        <v>5.937320984080647e-05</v>
       </c>
       <c r="O5" t="n">
-        <v>0.162990106648119</v>
+        <v>0.1341595742102636</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__learning_rate': 0.06385398733009987, 'model__loss': 'absolute_error', 'model__max_depth': 2, 'model__max_features': 'log2', 'model__min_samples_leaf': 18, 'model__min_samples_split': 12, 'model__n_estimators': 68, 'model__n_iter_no_change': 9, 'model__subsample': 0.7589322754697926, 'model__tol': 0.0008071612428512736, 'model__validation_fraction': 0.16299010664811903})</t>
+          <t>OrderedDict({'model__learning_rate': 0.061679538755918244, 'model__loss': 'huber', 'model__max_depth': 3, 'model__max_features': 'log2', 'model__min_samples_leaf': 13, 'model__min_samples_split': 13, 'model__n_estimators': 148, 'model__n_iter_no_change': 14, 'model__subsample': 0.8279822153767209, 'model__tol': 5.937320984080647e-05, 'model__validation_fraction': 0.13415957421026364})</t>
         </is>
       </c>
       <c r="Q5" t="n">
-        <v>0.5294460930779431</v>
+        <v>-0.04823091571603522</v>
       </c>
       <c r="R5" t="n">
-        <v>0.576015926496164</v>
+        <v>-0.2377612372449087</v>
       </c>
       <c r="S5" t="n">
-        <v>0.5527310097870535</v>
+        <v>-0.142996076480472</v>
       </c>
       <c r="T5" t="n">
-        <v>0.02328491670911043</v>
+        <v>0.09476516076443675</v>
       </c>
       <c r="U5" t="n">
         <v>4</v>
       </c>
       <c r="V5" t="n">
-        <v>0.5771672392095605</v>
+        <v>0.8138510099040869</v>
       </c>
       <c r="W5" t="n">
-        <v>0.5506617151058812</v>
+        <v>0.86305142858953</v>
       </c>
       <c r="X5" t="n">
-        <v>0.5639144771577209</v>
+        <v>0.8384512192468084</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.01325276205183962</v>
+        <v>0.02460020934272156</v>
       </c>
       <c r="Z5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.1258914470672607</v>
+        <v>0.3642693758010864</v>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>0.001763463020324707</v>
       </c>
       <c r="C6" t="n">
-        <v>0.005511283874511719</v>
+        <v>0.00901484489440918</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0004911422729492188</v>
+        <v>0.0005049705505371094</v>
       </c>
       <c r="E6" t="n">
-        <v>0.03705491779715134</v>
+        <v>0.06059114141190369</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>absolute_error</t>
+          <t>huber</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>sqrt</t>
+          <t>log2</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="J6" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="K6" t="n">
-        <v>70</v>
+        <v>105</v>
       </c>
       <c r="L6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="M6" t="n">
-        <v>0.7393351057584503</v>
+        <v>0.6882709613819928</v>
       </c>
       <c r="N6" t="n">
-        <v>0.0008839220247589657</v>
+        <v>0.0002083782840547887</v>
       </c>
       <c r="O6" t="n">
-        <v>0.1703467531106304</v>
+        <v>0.1512987949491055</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__learning_rate': 0.03705491779715134, 'model__loss': 'absolute_error', 'model__max_depth': 2, 'model__max_features': 'sqrt', 'model__min_samples_leaf': 8, 'model__min_samples_split': 24, 'model__n_estimators': 70, 'model__n_iter_no_change': 13, 'model__subsample': 0.7393351057584503, 'model__tol': 0.0008839220247589657, 'model__validation_fraction': 0.1703467531106304})</t>
+          <t>OrderedDict({'model__learning_rate': 0.060591141411903686, 'model__loss': 'huber', 'model__max_depth': 3, 'model__max_features': 'log2', 'model__min_samples_leaf': 19, 'model__min_samples_split': 32, 'model__n_estimators': 105, 'model__n_iter_no_change': 12, 'model__subsample': 0.6882709613819928, 'model__tol': 0.00020837828405478867, 'model__validation_fraction': 0.15129879494910548})</t>
         </is>
       </c>
       <c r="Q6" t="n">
-        <v>0.4815120558403544</v>
+        <v>-0.04591362345606687</v>
       </c>
       <c r="R6" t="n">
-        <v>0.5129271255605855</v>
+        <v>-0.3061455217506068</v>
       </c>
       <c r="S6" t="n">
-        <v>0.4972195907004699</v>
+        <v>-0.1760295726033368</v>
       </c>
       <c r="T6" t="n">
-        <v>0.01570753486011556</v>
+        <v>0.13011594914727</v>
       </c>
       <c r="U6" t="n">
         <v>5</v>
       </c>
       <c r="V6" t="n">
-        <v>0.5265622939996402</v>
+        <v>0.790306465389121</v>
       </c>
       <c r="W6" t="n">
-        <v>0.486650844357013</v>
+        <v>0.8404053281454666</v>
       </c>
       <c r="X6" t="n">
-        <v>0.5066065691783266</v>
+        <v>0.8153558967672938</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.01995572482131358</v>
+        <v>0.02504943137817284</v>
       </c>
       <c r="Z6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1709,41 +1709,41 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>numericals__mw_in</t>
+          <t>numericals__flowrate</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2450078064418788</v>
+        <v>0.2352725198289301</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>categoricals__bitsize_24</t>
+          <t>numericals__torque</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.208522719579171</v>
+        <v>0.1894447680608324</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>numericals__flowrate</t>
+          <t>numericals__mw_in</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1575151307922354</v>
+        <v>0.1805285919667912</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>numericals__torque</t>
+          <t>categoricals__bitsize_24</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.114906163127451</v>
+        <v>0.1403695714256666</v>
       </c>
     </row>
     <row r="6">
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.06812400088663097</v>
+        <v>0.1224224818983689</v>
       </c>
     </row>
     <row r="7">
@@ -1763,37 +1763,37 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.0624617866435629</v>
+        <v>0.05063178981602993</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>numericals__rpm</t>
+          <t>categoricals__bitsize_8.5</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.06101576768851236</v>
+        <v>0.0264549759383193</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>categoricals__bitsize_8.5</t>
+          <t>categoricals__bitsize_26</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.04429870245775066</v>
+        <v>0.02644799274995568</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>categoricals__bitsize_26</t>
+          <t>numericals__rpm</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.01836818120000118</v>
+        <v>0.02290943368290234</v>
       </c>
     </row>
     <row r="11">
@@ -1803,7 +1803,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.01427065385174072</v>
+        <v>0.004235067432554703</v>
       </c>
     </row>
     <row r="12">
@@ -1813,7 +1813,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.003021934570490006</v>
+        <v>0.001064337412161296</v>
       </c>
     </row>
     <row r="13">
@@ -1823,7 +1823,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.002487152760574977</v>
+        <v>0.0002184697874874659</v>
       </c>
     </row>
   </sheetData>
@@ -1864,10 +1864,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.3140396510564788</v>
+        <v>0.1613223328993759</v>
       </c>
       <c r="C2" t="n">
-        <v>0.009052246299831028</v>
+        <v>0.005533216057774872</v>
       </c>
     </row>
     <row r="3">
@@ -1877,75 +1877,75 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.2984284862054716</v>
+        <v>0.1606908419848764</v>
       </c>
       <c r="C3" t="n">
-        <v>0.008093088698375292</v>
+        <v>0.006485568455568777</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>torque</t>
+          <t>flowrate</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1326948044374564</v>
+        <v>0.06680247124761914</v>
       </c>
       <c r="C4" t="n">
-        <v>0.005744939292946883</v>
+        <v>0.002314489427219928</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>flowrate</t>
+          <t>torque</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.07496757027379189</v>
+        <v>0.06560902037585667</v>
       </c>
       <c r="C5" t="n">
-        <v>0.001690387556695311</v>
+        <v>0.004494251314625453</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>wob</t>
+          <t>spp</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.0669467876537244</v>
+        <v>0.026145558248158</v>
       </c>
       <c r="C6" t="n">
-        <v>0.002846894250896443</v>
+        <v>0.002782256316536296</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>rpm</t>
+          <t>wob</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.0491015924822408</v>
+        <v>0.01135725175349173</v>
       </c>
       <c r="C7" t="n">
-        <v>0.002767620900812734</v>
+        <v>0.0009875406782918201</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>spp</t>
+          <t>rpm</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.03825624948469868</v>
+        <v>0.008562465086034421</v>
       </c>
       <c r="C8" t="n">
-        <v>0.001465743547656875</v>
+        <v>0.0005614138268576655</v>
       </c>
     </row>
   </sheetData>
@@ -1959,21 +1959,139 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>message</t>
+          <t>feature</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>importance</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Additivity check failed in TreeExplainer! Please ensure the data matrix you passed to the explainer is the same shape that the model was trained on. If your data shape is correct then please report this on GitHub. This check failed because for one of the samples the sum of the SHAP values was 7.670325, while the model output was 7.828041. If this difference is acceptable you can set check_additivity=False to disable this check.</t>
-        </is>
+          <t>numericals__mw_in</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.6092608007275603</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>numericals__torque</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.5844097863220972</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>categoricals__bitsize_24</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.4832658763890992</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>numericals__flowrate</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.3970775308096567</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>numericals__spp</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.3005771202187278</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>numericals__wob</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.1272787398956481</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>numericals__rpm</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.07364627076663137</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>categoricals__bitsize_26</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.06899519536871034</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>categoricals__bitsize_8.5</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.05235795968008365</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>categoricals__bitsize_17</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.00652874654239964</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>categoricals__bitsize_12.25</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.004055998965288024</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>categoricals__bitsize_12</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.0005320151194295646</v>
       </c>
     </row>
   </sheetData>
@@ -2045,35 +2163,35 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__l2_regularization': 1.0889237550644373, 'model__learning_rate': 0.0696604761871229, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 596, 'model__max_leaf_nodes': 22, 'model__min_samples_leaf': 59, 'model__n_iter_no_change': 18, 'model__tol': 0.00029360602985208155, 'model__validation_fraction': 0.20245894424862895})</t>
+          <t>OrderedDict({'model__l2_regularization': 1.3143839143527278, 'model__learning_rate': 0.020000000000000004, 'model__loss': 'squared_error', 'model__max_depth': 2, 'model__max_iter': 300, 'model__max_leaf_nodes': 31, 'model__min_samples_leaf': 80, 'model__n_iter_no_change': 10, 'model__tol': 6.185326471010234e-05, 'model__validation_fraction': 0.25})</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8688782618292484</v>
+        <v>0.6750586454318424</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8435790319421856</v>
+        <v>0.5448982864179632</v>
       </c>
       <c r="D2" t="n">
-        <v>1.04025269998195</v>
+        <v>1.957518884701225</v>
       </c>
       <c r="E2" t="n">
-        <v>1.437247377164544</v>
+        <v>2.53601041030362</v>
       </c>
       <c r="F2" t="n">
-        <v>0.02529922988706279</v>
+        <v>0.1301603590138791</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8635426478146394</v>
+        <v>0.7588469253790955</v>
       </c>
       <c r="H2" t="n">
-        <v>0.7876187444750997</v>
+        <v>-0.07476905660647337</v>
       </c>
       <c r="I2" t="n">
-        <v>0.07592390333953969</v>
+        <v>0.8336159819855689</v>
       </c>
       <c r="J2" t="n">
-        <v>0.7496567928053299</v>
+        <v>-0.4915770475992578</v>
       </c>
     </row>
   </sheetData>
@@ -2229,22 +2347,22 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.3339356184005737</v>
+        <v>0.1146632432937622</v>
       </c>
       <c r="B2" t="n">
-        <v>0.003346800804138184</v>
+        <v>0.001499295234680176</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1196006536483765</v>
+        <v>0.04552102088928223</v>
       </c>
       <c r="D2" t="n">
-        <v>0.001170754432678223</v>
+        <v>0.0005002021789550781</v>
       </c>
       <c r="E2" t="n">
-        <v>0.01</v>
+        <v>1.314383914352728</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1</v>
+        <v>0.02</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -2252,86 +2370,86 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I2" t="n">
-        <v>486</v>
+        <v>300</v>
       </c>
       <c r="J2" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="K2" t="n">
+        <v>80</v>
+      </c>
+      <c r="L2" t="n">
+        <v>10</v>
+      </c>
+      <c r="M2" t="n">
+        <v>6.185326471010234e-05</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>OrderedDict({'model__l2_regularization': 1.3143839143527278, 'model__learning_rate': 0.020000000000000004, 'model__loss': 'squared_error', 'model__max_depth': 2, 'model__max_iter': 300, 'model__max_leaf_nodes': 31, 'model__min_samples_leaf': 80, 'model__n_iter_no_change': 10, 'model__tol': 6.185326471010234e-05, 'model__validation_fraction': 0.25})</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>0.01065233194125881</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>-0.1601904451542056</v>
+      </c>
+      <c r="R2" t="n">
+        <v>-0.07476905660647337</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.08542138854773218</v>
+      </c>
+      <c r="T2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.7375837422586177</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.7801101084995732</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0.7588469253790955</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0.02126318312047776</v>
+      </c>
+      <c r="Y2" t="n">
         <v>20</v>
       </c>
-      <c r="L2" t="n">
-        <v>30</v>
-      </c>
-      <c r="M2" t="n">
-        <v>2.221256745984293e-05</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.126647090810371</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>OrderedDict({'model__l2_regularization': 0.01, 'model__learning_rate': 0.1, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 486, 'model__max_leaf_nodes': 27, 'model__min_samples_leaf': 20, 'model__n_iter_no_change': 30, 'model__tol': 2.2212567459842933e-05, 'model__validation_fraction': 0.126647090810371})</t>
-        </is>
-      </c>
-      <c r="P2" t="n">
-        <v>0.8047953100192038</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0.8248688184228374</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0.8148320642210206</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0.01003675420181682</v>
-      </c>
-      <c r="T2" t="n">
-        <v>2</v>
-      </c>
-      <c r="U2" t="n">
-        <v>0.9186177879498595</v>
-      </c>
-      <c r="V2" t="n">
-        <v>0.9148307600680624</v>
-      </c>
-      <c r="W2" t="n">
-        <v>0.9167242740089609</v>
-      </c>
-      <c r="X2" t="n">
-        <v>0.001893513940898539</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>3</v>
-      </c>
       <c r="Z2" t="n">
-        <v>0.1018922097879403</v>
+        <v>0.8336159819855689</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.7638859593270504</v>
+        <v>-0.4915770475992578</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.5843136310577393</v>
+        <v>0.2314621210098267</v>
       </c>
       <c r="B3" t="n">
-        <v>0.005838632583618164</v>
+        <v>0.001003384590148926</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2366670370101929</v>
+        <v>0.08555924892425537</v>
       </c>
       <c r="D3" t="n">
-        <v>0.003358960151672363</v>
+        <v>0.001000761985778809</v>
       </c>
       <c r="E3" t="n">
-        <v>20</v>
+        <v>0.01</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1</v>
+        <v>0.02</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2342,83 +2460,83 @@
         <v>4</v>
       </c>
       <c r="I3" t="n">
-        <v>800</v>
+        <v>300</v>
       </c>
       <c r="J3" t="n">
+        <v>8</v>
+      </c>
+      <c r="K3" t="n">
+        <v>80</v>
+      </c>
+      <c r="L3" t="n">
+        <v>10</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>OrderedDict({'model__l2_regularization': 0.01, 'model__learning_rate': 0.020000000000000004, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 300, 'model__max_leaf_nodes': 8, 'model__min_samples_leaf': 80, 'model__n_iter_no_change': 10, 'model__tol': 0.001, 'model__validation_fraction': 0.25})</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>0.02563726014117884</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>-0.2353697801038552</v>
+      </c>
+      <c r="R3" t="n">
+        <v>-0.1048662599813382</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.130503520122517</v>
+      </c>
+      <c r="T3" t="n">
+        <v>2</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.7927098845940505</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.8432835320467602</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.8179967083204054</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0.02528682372635488</v>
+      </c>
+      <c r="Y3" t="n">
         <v>18</v>
       </c>
-      <c r="K3" t="n">
-        <v>20</v>
-      </c>
-      <c r="L3" t="n">
-        <v>30</v>
-      </c>
-      <c r="M3" t="n">
-        <v>1e-05</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>OrderedDict({'model__l2_regularization': 20.0, 'model__learning_rate': 0.1, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 800, 'model__max_leaf_nodes': 18, 'model__min_samples_leaf': 20, 'model__n_iter_no_change': 30, 'model__tol': 1e-05, 'model__validation_fraction': 0.12})</t>
-        </is>
-      </c>
-      <c r="P3" t="n">
-        <v>0.8099998508742233</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0.8258569284143015</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0.8179283896442624</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0.007928538770039073</v>
-      </c>
-      <c r="T3" t="n">
-        <v>1</v>
-      </c>
-      <c r="U3" t="n">
-        <v>0.9287318415937431</v>
-      </c>
-      <c r="V3" t="n">
-        <v>0.923477707947037</v>
-      </c>
-      <c r="W3" t="n">
-        <v>0.9261047747703901</v>
-      </c>
-      <c r="X3" t="n">
-        <v>0.002627066823353064</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>1</v>
-      </c>
       <c r="Z3" t="n">
-        <v>0.1081763851261277</v>
+        <v>0.9228629683017435</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.7638401970811985</v>
+        <v>-0.5662977441322099</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.5481331348419189</v>
+        <v>0.3559632301330566</v>
       </c>
       <c r="B4" t="n">
-        <v>0.05568647384643555</v>
+        <v>0.003499984741210938</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1812098026275635</v>
+        <v>0.1087048053741455</v>
       </c>
       <c r="D4" t="n">
-        <v>0.01535224914550781</v>
+        <v>0.00249934196472168</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01</v>
+        <v>20</v>
       </c>
       <c r="F4" t="n">
-        <v>0.06338434660149135</v>
+        <v>0.02361507782876152</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -2429,83 +2547,83 @@
         <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>800</v>
+        <v>300</v>
       </c>
       <c r="J4" t="n">
         <v>31</v>
       </c>
       <c r="K4" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="L4" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="M4" t="n">
-        <v>0.001</v>
+        <v>1e-05</v>
       </c>
       <c r="N4" t="n">
-        <v>0.12</v>
+        <v>0.25</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__l2_regularization': 0.01, 'model__learning_rate': 0.06338434660149135, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 800, 'model__max_leaf_nodes': 31, 'model__min_samples_leaf': 20, 'model__n_iter_no_change': 30, 'model__tol': 0.001, 'model__validation_fraction': 0.12})</t>
+          <t>OrderedDict({'model__l2_regularization': 20.0, 'model__learning_rate': 0.023615077828761516, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 300, 'model__max_leaf_nodes': 31, 'model__min_samples_leaf': 80, 'model__n_iter_no_change': 10, 'model__tol': 1e-05, 'model__validation_fraction': 0.25})</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>0.8009735179318818</v>
+        <v>0.03410986536323179</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.8237081163421227</v>
+        <v>-0.2508416103883708</v>
       </c>
       <c r="R4" t="n">
-        <v>0.8123408171370022</v>
+        <v>-0.1083658725125695</v>
       </c>
       <c r="S4" t="n">
-        <v>0.01136729920512047</v>
+        <v>0.1424757378758013</v>
       </c>
       <c r="T4" t="n">
         <v>3</v>
       </c>
       <c r="U4" t="n">
-        <v>0.9146014440059603</v>
+        <v>0.8014168428501024</v>
       </c>
       <c r="V4" t="n">
-        <v>0.9200818322609494</v>
+        <v>0.84955152793408</v>
       </c>
       <c r="W4" t="n">
-        <v>0.9173416381334549</v>
+        <v>0.8254841853920911</v>
       </c>
       <c r="X4" t="n">
-        <v>0.002740194127494544</v>
+        <v>0.02406734254198878</v>
       </c>
       <c r="Y4" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.1050008209964527</v>
+        <v>0.9338500579046607</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.7598404066387758</v>
+        <v>-0.5752909014648999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.450284481048584</v>
+        <v>0.1631022691726685</v>
       </c>
       <c r="B5" t="n">
-        <v>0.001999616622924805</v>
+        <v>0.002255558967590332</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1865460872650146</v>
+        <v>0.06855762004852295</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0005011558532714844</v>
+        <v>0.0009974241256713867</v>
       </c>
       <c r="E5" t="n">
         <v>20</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1</v>
+        <v>0.03026775896411537</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -2513,86 +2631,86 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I5" t="n">
-        <v>800</v>
+        <v>440</v>
       </c>
       <c r="J5" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="K5" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="L5" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="M5" t="n">
         <v>1e-05</v>
       </c>
       <c r="N5" t="n">
-        <v>0.12</v>
+        <v>0.25</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__l2_regularization': 20.0, 'model__learning_rate': 0.1, 'model__loss': 'squared_error', 'model__max_depth': 3, 'model__max_iter': 800, 'model__max_leaf_nodes': 8, 'model__min_samples_leaf': 20, 'model__n_iter_no_change': 30, 'model__tol': 1e-05, 'model__validation_fraction': 0.12})</t>
+          <t>OrderedDict({'model__l2_regularization': 20.0, 'model__learning_rate': 0.03026775896411537, 'model__loss': 'squared_error', 'model__max_depth': 2, 'model__max_iter': 440, 'model__max_leaf_nodes': 24, 'model__min_samples_leaf': 80, 'model__n_iter_no_change': 10, 'model__tol': 1e-05, 'model__validation_fraction': 0.25})</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>0.7928493086831504</v>
+        <v>0.01268992233509492</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.8117269334356478</v>
+        <v>-0.2670882543601796</v>
       </c>
       <c r="R5" t="n">
-        <v>0.8022881210593991</v>
+        <v>-0.1271991660125423</v>
       </c>
       <c r="S5" t="n">
-        <v>0.009438812376248717</v>
+        <v>0.1398890883476372</v>
       </c>
       <c r="T5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U5" t="n">
-        <v>0.8944091194873957</v>
+        <v>0.7697899818908974</v>
       </c>
       <c r="V5" t="n">
-        <v>0.8876266427784656</v>
+        <v>0.8216888747120333</v>
       </c>
       <c r="W5" t="n">
-        <v>0.8910178811329306</v>
+        <v>0.7957394283014654</v>
       </c>
       <c r="X5" t="n">
-        <v>0.003391238354465032</v>
+        <v>0.02594944641056796</v>
       </c>
       <c r="Y5" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.08872976007353151</v>
+        <v>0.9229385943140077</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.7579232410226333</v>
+        <v>-0.5886684631695462</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.424923300743103</v>
+        <v>0.1668182611465454</v>
       </c>
       <c r="B6" t="n">
-        <v>0.003847241401672363</v>
+        <v>0.001021504402160645</v>
       </c>
       <c r="C6" t="n">
-        <v>0.1613248586654663</v>
+        <v>0.06306111812591553</v>
       </c>
       <c r="D6" t="n">
-        <v>0.001294255256652832</v>
+        <v>0.001006245613098145</v>
       </c>
       <c r="E6" t="n">
-        <v>0.01</v>
+        <v>0.1504850684084423</v>
       </c>
       <c r="F6" t="n">
-        <v>0.06069782862764342</v>
+        <v>0.02051854371502429</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -2600,86 +2718,86 @@
         </is>
       </c>
       <c r="H6" t="n">
+        <v>3</v>
+      </c>
+      <c r="I6" t="n">
+        <v>306</v>
+      </c>
+      <c r="J6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K6" t="n">
+        <v>23</v>
+      </c>
+      <c r="L6" t="n">
+        <v>10</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1.237464367747911e-05</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.2454249620131051</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>OrderedDict({'model__l2_regularization': 0.15048506840844234, 'model__learning_rate': 0.020518543715024287, 'model__loss': 'squared_error', 'model__max_depth': 3, 'model__max_iter': 306, 'model__max_leaf_nodes': 18, 'model__min_samples_leaf': 23, 'model__n_iter_no_change': 10, 'model__tol': 1.237464367747911e-05, 'model__validation_fraction': 0.24542496201310512})</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>0.03022393124647871</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>-0.2681196779482087</v>
+      </c>
+      <c r="R6" t="n">
+        <v>-0.118947873350865</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0.1491718045973437</v>
+      </c>
+      <c r="T6" t="n">
         <v>4</v>
       </c>
-      <c r="I6" t="n">
-        <v>800</v>
-      </c>
-      <c r="J6" t="n">
-        <v>9</v>
-      </c>
-      <c r="K6" t="n">
-        <v>20</v>
-      </c>
-      <c r="L6" t="n">
-        <v>30</v>
-      </c>
-      <c r="M6" t="n">
-        <v>1e-05</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>OrderedDict({'model__l2_regularization': 0.01, 'model__learning_rate': 0.06069782862764342, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 800, 'model__max_leaf_nodes': 9, 'model__min_samples_leaf': 20, 'model__n_iter_no_change': 30, 'model__tol': 1e-05, 'model__validation_fraction': 0.25})</t>
-        </is>
-      </c>
-      <c r="P6" t="n">
-        <v>0.786737759094111</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0.8090659696359114</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0.7979018643650112</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0.01116410527090017</v>
-      </c>
-      <c r="T6" t="n">
-        <v>6</v>
-      </c>
       <c r="U6" t="n">
-        <v>0.886682628718465</v>
+        <v>0.800765408421741</v>
       </c>
       <c r="V6" t="n">
-        <v>0.8802277147594062</v>
+        <v>0.8473428917708186</v>
       </c>
       <c r="W6" t="n">
-        <v>0.8834551717389356</v>
+        <v>0.8240541500962798</v>
       </c>
       <c r="X6" t="n">
-        <v>0.003227456979529419</v>
+        <v>0.02328874167453876</v>
       </c>
       <c r="Y6" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.08555330737392441</v>
+        <v>0.9430020234471448</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.7551252106780491</v>
+        <v>-0.5904488850744374</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.347252368927002</v>
+        <v>0.1947795152664185</v>
       </c>
       <c r="B7" t="n">
-        <v>0.01288580894470215</v>
+        <v>0.00184786319732666</v>
       </c>
       <c r="C7" t="n">
-        <v>0.1375417709350586</v>
+        <v>0.07503998279571533</v>
       </c>
       <c r="D7" t="n">
-        <v>0.003268003463745117</v>
+        <v>0.0002034902572631836</v>
       </c>
       <c r="E7" t="n">
-        <v>5.810909071553644</v>
+        <v>20</v>
       </c>
       <c r="F7" t="n">
-        <v>0.08287830852695076</v>
+        <v>0.02</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -2690,83 +2808,83 @@
         <v>4</v>
       </c>
       <c r="I7" t="n">
-        <v>732</v>
+        <v>300</v>
       </c>
       <c r="J7" t="n">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="K7" t="n">
-        <v>28</v>
+        <v>80</v>
       </c>
       <c r="L7" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0001868349859728154</v>
+        <v>0.0001983923984405631</v>
       </c>
       <c r="N7" t="n">
-        <v>0.2439524195246732</v>
+        <v>0.12</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__l2_regularization': 5.8109090715536444, 'model__learning_rate': 0.08287830852695076, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 732, 'model__max_leaf_nodes': 9, 'model__min_samples_leaf': 28, 'model__n_iter_no_change': 17, 'model__tol': 0.00018683498597281536, 'model__validation_fraction': 0.24395241952467317})</t>
+          <t>OrderedDict({'model__l2_regularization': 20.0, 'model__learning_rate': 0.020000000000000004, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 300, 'model__max_leaf_nodes': 31, 'model__min_samples_leaf': 80, 'model__n_iter_no_change': 10, 'model__tol': 0.00019839239844056308, 'model__validation_fraction': 0.12})</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>0.7830967555933808</v>
+        <v>0.01132505315818033</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.8056657833855859</v>
+        <v>-0.25619836212875</v>
       </c>
       <c r="R7" t="n">
-        <v>0.7943812694894834</v>
+        <v>-0.1224366544852848</v>
       </c>
       <c r="S7" t="n">
-        <v>0.01128451389610258</v>
+        <v>0.1337617076434652</v>
       </c>
       <c r="T7" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U7" t="n">
-        <v>0.8839190213928227</v>
+        <v>0.8044363611263217</v>
       </c>
       <c r="V7" t="n">
-        <v>0.8724277136907576</v>
+        <v>0.8496858952242466</v>
       </c>
       <c r="W7" t="n">
-        <v>0.8781733675417902</v>
+        <v>0.8270611281752842</v>
       </c>
       <c r="X7" t="n">
-        <v>0.005745653851032595</v>
+        <v>0.02262476704896249</v>
       </c>
       <c r="Y7" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.08379209805230681</v>
+        <v>0.9494977826605691</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.75248522046333</v>
+        <v>-0.5971855458155694</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.3820804357528687</v>
+        <v>0.1874054670333862</v>
       </c>
       <c r="B8" t="n">
-        <v>0.01687777042388916</v>
+        <v>3.457069396972656e-06</v>
       </c>
       <c r="C8" t="n">
-        <v>0.1562302112579346</v>
+        <v>0.07230055332183838</v>
       </c>
       <c r="D8" t="n">
-        <v>0.005888223648071289</v>
+        <v>0.001754641532897949</v>
       </c>
       <c r="E8" t="n">
-        <v>1.088923755064437</v>
+        <v>0.01</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0696604761871229</v>
+        <v>0.03108684446665815</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -2777,83 +2895,83 @@
         <v>4</v>
       </c>
       <c r="I8" t="n">
-        <v>596</v>
+        <v>300</v>
       </c>
       <c r="J8" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="K8" t="n">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="L8" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0002936060298520815</v>
+        <v>0.001</v>
       </c>
       <c r="N8" t="n">
-        <v>0.202458944248629</v>
+        <v>0.25</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__l2_regularization': 1.0889237550644373, 'model__learning_rate': 0.0696604761871229, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 596, 'model__max_leaf_nodes': 22, 'model__min_samples_leaf': 59, 'model__n_iter_no_change': 18, 'model__tol': 0.00029360602985208155, 'model__validation_fraction': 0.20245894424862895})</t>
+          <t>OrderedDict({'model__l2_regularization': 0.01, 'model__learning_rate': 0.03108684446665815, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 300, 'model__max_leaf_nodes': 31, 'model__min_samples_leaf': 80, 'model__n_iter_no_change': 10, 'model__tol': 0.001, 'model__validation_fraction': 0.25})</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0.7809315819210253</v>
+        <v>0.01362358093375926</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.7943059070291741</v>
+        <v>-0.3144024154125085</v>
       </c>
       <c r="R8" t="n">
-        <v>0.7876187444750997</v>
+        <v>-0.1503894172393746</v>
       </c>
       <c r="S8" t="n">
-        <v>0.006687162554074422</v>
+        <v>0.1640129981731339</v>
       </c>
       <c r="T8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U8" t="n">
-        <v>0.87007136053342</v>
+        <v>0.8209051924455129</v>
       </c>
       <c r="V8" t="n">
-        <v>0.8570139350958588</v>
+        <v>0.8630915159147228</v>
       </c>
       <c r="W8" t="n">
-        <v>0.8635426478146394</v>
+        <v>0.8419983541801178</v>
       </c>
       <c r="X8" t="n">
-        <v>0.006528712718780638</v>
+        <v>0.02109316173460496</v>
       </c>
       <c r="Y8" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.07592390333953969</v>
+        <v>0.9923877714194924</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.7496567928053299</v>
+        <v>-0.6465833029491208</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.4513814449310303</v>
+        <v>0.1905121803283691</v>
       </c>
       <c r="B9" t="n">
-        <v>0.07918858528137207</v>
+        <v>0.001992464065551758</v>
       </c>
       <c r="C9" t="n">
-        <v>0.1467511653900146</v>
+        <v>0.07844674587249756</v>
       </c>
       <c r="D9" t="n">
-        <v>0.02240276336669922</v>
+        <v>0.0003353357315063477</v>
       </c>
       <c r="E9" t="n">
-        <v>0.01</v>
+        <v>20</v>
       </c>
       <c r="F9" t="n">
-        <v>0.1</v>
+        <v>0.03342652505864618</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -2864,83 +2982,83 @@
         <v>4</v>
       </c>
       <c r="I9" t="n">
-        <v>686</v>
+        <v>326</v>
       </c>
       <c r="J9" t="n">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="K9" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="L9" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="M9" t="n">
-        <v>0.001</v>
+        <v>0.0002587540924911034</v>
       </c>
       <c r="N9" t="n">
-        <v>0.25</v>
+        <v>0.1676022884240263</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__l2_regularization': 0.01, 'model__learning_rate': 0.1, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 686, 'model__max_leaf_nodes': 31, 'model__min_samples_leaf': 20, 'model__n_iter_no_change': 30, 'model__tol': 0.001, 'model__validation_fraction': 0.25})</t>
+          <t>OrderedDict({'model__l2_regularization': 20.0, 'model__learning_rate': 0.03342652505864618, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 326, 'model__max_leaf_nodes': 12, 'model__min_samples_leaf': 80, 'model__n_iter_no_change': 22, 'model__tol': 0.0002587540924911034, 'model__validation_fraction': 0.1676022884240263})</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>0.7876735930921346</v>
+        <v>0.006841865026382399</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.8179558590449543</v>
+        <v>-0.3235293591756854</v>
       </c>
       <c r="R9" t="n">
-        <v>0.8028147260685444</v>
+        <v>-0.1583437470746515</v>
       </c>
       <c r="S9" t="n">
-        <v>0.01514113297640984</v>
+        <v>0.1651856121010339</v>
       </c>
       <c r="T9" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="U9" t="n">
-        <v>0.9051257192657933</v>
+        <v>0.823958318880629</v>
       </c>
       <c r="V9" t="n">
-        <v>0.9137466431184426</v>
+        <v>0.8679132352886664</v>
       </c>
       <c r="W9" t="n">
-        <v>0.9094361811921179</v>
+        <v>0.8459357770846476</v>
       </c>
       <c r="X9" t="n">
-        <v>0.004310461926324616</v>
+        <v>0.0219774582040187</v>
       </c>
       <c r="Y9" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.1066214551235735</v>
+        <v>1.004279524159299</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.7495039985067578</v>
+        <v>-0.660483509154301</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.2263858318328857</v>
+        <v>0.2350952625274658</v>
       </c>
       <c r="B10" t="n">
-        <v>0.04837703704833984</v>
+        <v>0.002758264541625977</v>
       </c>
       <c r="C10" t="n">
-        <v>0.07317125797271729</v>
+        <v>0.08131611347198486</v>
       </c>
       <c r="D10" t="n">
-        <v>0.01562631130218506</v>
+        <v>0.001245379447937012</v>
       </c>
       <c r="E10" t="n">
-        <v>0.01</v>
+        <v>20</v>
       </c>
       <c r="F10" t="n">
-        <v>0.06406748845753643</v>
+        <v>0.02666083832803979</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -2951,7 +3069,7 @@
         <v>4</v>
       </c>
       <c r="I10" t="n">
-        <v>800</v>
+        <v>300</v>
       </c>
       <c r="J10" t="n">
         <v>31</v>
@@ -2963,71 +3081,71 @@
         <v>10</v>
       </c>
       <c r="M10" t="n">
-        <v>0.001</v>
+        <v>1.649822069540698e-05</v>
       </c>
       <c r="N10" t="n">
-        <v>0.12</v>
+        <v>0.1485559334972484</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__l2_regularization': 0.01, 'model__learning_rate': 0.06406748845753643, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 800, 'model__max_leaf_nodes': 31, 'model__min_samples_leaf': 20, 'model__n_iter_no_change': 10, 'model__tol': 0.001, 'model__validation_fraction': 0.12})</t>
+          <t>OrderedDict({'model__l2_regularization': 20.0, 'model__learning_rate': 0.026660838328039792, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 300, 'model__max_leaf_nodes': 31, 'model__min_samples_leaf': 20, 'model__n_iter_no_change': 10, 'model__tol': 1.649822069540698e-05, 'model__validation_fraction': 0.14855593349724838})</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>0.7712867191800434</v>
+        <v>-0.04698670712388209</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.8013714442226393</v>
+        <v>-0.299789741871928</v>
       </c>
       <c r="R10" t="n">
-        <v>0.7863290817013413</v>
+        <v>-0.173388224497905</v>
       </c>
       <c r="S10" t="n">
-        <v>0.01504236252129793</v>
+        <v>0.1264015173740229</v>
       </c>
       <c r="T10" t="n">
         <v>9</v>
       </c>
       <c r="U10" t="n">
-        <v>0.8537366074584102</v>
+        <v>0.8428995940223465</v>
       </c>
       <c r="V10" t="n">
-        <v>0.8748216121077419</v>
+        <v>0.8837318788626901</v>
       </c>
       <c r="W10" t="n">
-        <v>0.864279109783076</v>
+        <v>0.8633157364425184</v>
       </c>
       <c r="X10" t="n">
-        <v>0.01054250232466586</v>
+        <v>0.02041614242017181</v>
       </c>
       <c r="Y10" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.07795002808173468</v>
+        <v>1.036703960940423</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.747354067660474</v>
+        <v>-0.6917402049681167</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.2797772884368896</v>
+        <v>0.3917664289474487</v>
       </c>
       <c r="B11" t="n">
-        <v>0.05957150459289551</v>
+        <v>0.002549529075622559</v>
       </c>
       <c r="C11" t="n">
-        <v>0.100628137588501</v>
+        <v>0.1496142148971558</v>
       </c>
       <c r="D11" t="n">
-        <v>0.01753616333007812</v>
+        <v>0.0005480051040649414</v>
       </c>
       <c r="E11" t="n">
-        <v>2.736958202925582</v>
+        <v>4.80555470976749</v>
       </c>
       <c r="F11" t="n">
-        <v>0.08935348299163301</v>
+        <v>0.02637321417594226</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -3038,83 +3156,83 @@
         <v>4</v>
       </c>
       <c r="I11" t="n">
-        <v>790</v>
+        <v>562</v>
       </c>
       <c r="J11" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K11" t="n">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="L11" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="M11" t="n">
-        <v>6.277757293238185e-05</v>
+        <v>0.0006665883558488896</v>
       </c>
       <c r="N11" t="n">
-        <v>0.1757777063541278</v>
+        <v>0.1702833843482989</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__l2_regularization': 2.736958202925582, 'model__learning_rate': 0.08935348299163301, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 790, 'model__max_leaf_nodes': 15, 'model__min_samples_leaf': 74, 'model__n_iter_no_change': 19, 'model__tol': 6.277757293238185e-05, 'model__validation_fraction': 0.1757777063541278})</t>
+          <t>OrderedDict({'model__l2_regularization': 4.80555470976749, 'model__learning_rate': 0.026373214175942256, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 562, 'model__max_leaf_nodes': 10, 'model__min_samples_leaf': 65, 'model__n_iter_no_change': 27, 'model__tol': 0.0006665883558488896, 'model__validation_fraction': 0.17028338434829887})</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>0.7813521233295209</v>
+        <v>-0.06114264111542989</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.779541634078657</v>
+        <v>-0.3136748042641999</v>
       </c>
       <c r="R11" t="n">
-        <v>0.7804468787040889</v>
+        <v>-0.1874087226898149</v>
       </c>
       <c r="S11" t="n">
-        <v>0.0009052446254319557</v>
+        <v>0.126266081574385</v>
       </c>
       <c r="T11" t="n">
+        <v>10</v>
+      </c>
+      <c r="U11" t="n">
+        <v>0.850377543349606</v>
+      </c>
+      <c r="V11" t="n">
+        <v>0.8890113068603868</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0.8696944251049964</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0.01931688175539037</v>
+      </c>
+      <c r="Y11" t="n">
         <v>11</v>
       </c>
-      <c r="U11" t="n">
-        <v>0.8635263631602281</v>
-      </c>
-      <c r="V11" t="n">
-        <v>0.8301810040092494</v>
-      </c>
-      <c r="W11" t="n">
-        <v>0.8468536835847388</v>
-      </c>
-      <c r="X11" t="n">
-        <v>0.01667267957548935</v>
-      </c>
-      <c r="Y11" t="n">
-        <v>12</v>
-      </c>
       <c r="Z11" t="n">
-        <v>0.06640680488064987</v>
+        <v>1.057103147794811</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.747243476263764</v>
+        <v>-0.7159602965872205</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.3247330188751221</v>
+        <v>0.4491758346557617</v>
       </c>
       <c r="B12" t="n">
-        <v>0.002815723419189453</v>
+        <v>0.0314018726348877</v>
       </c>
       <c r="C12" t="n">
-        <v>0.1344610452651978</v>
+        <v>0.1782795190811157</v>
       </c>
       <c r="D12" t="n">
-        <v>0.001690506935119629</v>
+        <v>0.006321549415588379</v>
       </c>
       <c r="E12" t="n">
-        <v>0.01027977840987963</v>
+        <v>20</v>
       </c>
       <c r="F12" t="n">
-        <v>0.07458794605542038</v>
+        <v>0.0286382818879035</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -3122,86 +3240,86 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I12" t="n">
-        <v>589</v>
+        <v>800</v>
       </c>
       <c r="J12" t="n">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="K12" t="n">
-        <v>39</v>
+        <v>80</v>
       </c>
       <c r="L12" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="M12" t="n">
-        <v>0.0006133044588437132</v>
+        <v>0.0009851275402512813</v>
       </c>
       <c r="N12" t="n">
-        <v>0.2257260703867113</v>
+        <v>0.12</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__l2_regularization': 0.010279778409879632, 'model__learning_rate': 0.07458794605542038, 'model__loss': 'squared_error', 'model__max_depth': 3, 'model__max_iter': 589, 'model__max_leaf_nodes': 14, 'model__min_samples_leaf': 39, 'model__n_iter_no_change': 13, 'model__tol': 0.0006133044588437132, 'model__validation_fraction': 0.22572607038671127})</t>
+          <t>OrderedDict({'model__l2_regularization': 20.0, 'model__learning_rate': 0.028638281887903502, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 800, 'model__max_leaf_nodes': 31, 'model__min_samples_leaf': 80, 'model__n_iter_no_change': 10, 'model__tol': 0.0009851275402512813, 'model__validation_fraction': 0.12})</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>0.7675390103600814</v>
+        <v>-0.02615227905598649</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.7936976924848778</v>
+        <v>-0.3548962448129689</v>
       </c>
       <c r="R12" t="n">
-        <v>0.7806183514224796</v>
+        <v>-0.1905242619344777</v>
       </c>
       <c r="S12" t="n">
-        <v>0.01307934106239816</v>
+        <v>0.1643719828784912</v>
       </c>
       <c r="T12" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="U12" t="n">
-        <v>0.8531975803331904</v>
+        <v>0.8653182942574847</v>
       </c>
       <c r="V12" t="n">
-        <v>0.8475852795439328</v>
+        <v>0.8915919212114701</v>
       </c>
       <c r="W12" t="n">
-        <v>0.8503914299385615</v>
+        <v>0.8784551077344774</v>
       </c>
       <c r="X12" t="n">
-        <v>0.002806150394628781</v>
+        <v>0.01313681347699269</v>
       </c>
       <c r="Y12" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.06977307851608194</v>
+        <v>1.068979369668955</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.7457318121644386</v>
+        <v>-0.7250139467689553</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.2773244380950928</v>
+        <v>0.3976404666900635</v>
       </c>
       <c r="B13" t="n">
-        <v>0.0005006790161132812</v>
+        <v>0.01104164123535156</v>
       </c>
       <c r="C13" t="n">
-        <v>0.1104291677474976</v>
+        <v>0.1549115180969238</v>
       </c>
       <c r="D13" t="n">
-        <v>0.00100553035736084</v>
+        <v>0.001976728439331055</v>
       </c>
       <c r="E13" t="n">
-        <v>14.25809463775946</v>
+        <v>4.358628897525027</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0617651314239038</v>
+        <v>0.04047615571540435</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -3212,83 +3330,83 @@
         <v>3</v>
       </c>
       <c r="I13" t="n">
-        <v>491</v>
+        <v>752</v>
       </c>
       <c r="J13" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="K13" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="L13" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="M13" t="n">
-        <v>0.0001544393009519414</v>
+        <v>5.083556924570688e-05</v>
       </c>
       <c r="N13" t="n">
-        <v>0.1428678327264134</v>
+        <v>0.2057254097308825</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__l2_regularization': 14.258094637759456, 'model__learning_rate': 0.0617651314239038, 'model__loss': 'squared_error', 'model__max_depth': 3, 'model__max_iter': 491, 'model__max_leaf_nodes': 13, 'model__min_samples_leaf': 20, 'model__n_iter_no_change': 17, 'model__tol': 0.00015443930095194143, 'model__validation_fraction': 0.1428678327264134})</t>
+          <t>OrderedDict({'model__l2_regularization': 4.358628897525027, 'model__learning_rate': 0.040476155715404354, 'model__loss': 'squared_error', 'model__max_depth': 3, 'model__max_iter': 752, 'model__max_leaf_nodes': 24, 'model__min_samples_leaf': 45, 'model__n_iter_no_change': 23, 'model__tol': 5.083556924570688e-05, 'model__validation_fraction': 0.20572540973088252})</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>0.7673007883713283</v>
+        <v>-0.02040718817740195</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.7813958123473821</v>
+        <v>-0.3860069938356145</v>
       </c>
       <c r="R13" t="n">
-        <v>0.7743483003593552</v>
+        <v>-0.2032070910065082</v>
       </c>
       <c r="S13" t="n">
-        <v>0.007047511988026889</v>
+        <v>0.1827999028291063</v>
       </c>
       <c r="T13" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="U13" t="n">
-        <v>0.8410587509696139</v>
+        <v>0.8593247772274357</v>
       </c>
       <c r="V13" t="n">
-        <v>0.8264127451757499</v>
+        <v>0.9046380153984707</v>
       </c>
       <c r="W13" t="n">
-        <v>0.8337357480726819</v>
+        <v>0.8819813963129532</v>
       </c>
       <c r="X13" t="n">
-        <v>0.007323002896931996</v>
+        <v>0.02265661908551747</v>
       </c>
       <c r="Y13" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.05938744771332671</v>
+        <v>1.085188487319461</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.7446545765026918</v>
+        <v>-0.745801334666239</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0.3575927019119263</v>
+        <v>0.3505364656448364</v>
       </c>
       <c r="B14" t="n">
-        <v>0.001045584678649902</v>
+        <v>0.009859919548034668</v>
       </c>
       <c r="C14" t="n">
-        <v>0.1368743181228638</v>
+        <v>0.1351327896118164</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0005460977554321289</v>
+        <v>0.001709938049316406</v>
       </c>
       <c r="E14" t="n">
-        <v>0.2258215944659482</v>
+        <v>0.01027977840987963</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0645191239031175</v>
+        <v>0.07458794605542038</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -3299,83 +3417,83 @@
         <v>3</v>
       </c>
       <c r="I14" t="n">
-        <v>635</v>
+        <v>589</v>
       </c>
       <c r="J14" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="K14" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="L14" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="M14" t="n">
-        <v>4.063746627400014e-05</v>
+        <v>0.0006133044588437132</v>
       </c>
       <c r="N14" t="n">
-        <v>0.2042129064850941</v>
+        <v>0.2257260703867113</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__l2_regularization': 0.22582159446594824, 'model__learning_rate': 0.0645191239031175, 'model__loss': 'squared_error', 'model__max_depth': 3, 'model__max_iter': 635, 'model__max_leaf_nodes': 18, 'model__min_samples_leaf': 41, 'model__n_iter_no_change': 25, 'model__tol': 4.063746627400014e-05, 'model__validation_fraction': 0.2042129064850941})</t>
+          <t>OrderedDict({'model__l2_regularization': 0.010279778409879632, 'model__learning_rate': 0.07458794605542038, 'model__loss': 'squared_error', 'model__max_depth': 3, 'model__max_iter': 589, 'model__max_leaf_nodes': 14, 'model__min_samples_leaf': 39, 'model__n_iter_no_change': 13, 'model__tol': 0.0006133044588437132, 'model__validation_fraction': 0.22572607038671127})</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>0.7667278062634574</v>
+        <v>-0.03522527309899792</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.7904553568498452</v>
+        <v>-0.4338031984764594</v>
       </c>
       <c r="R14" t="n">
-        <v>0.7785915815566513</v>
+        <v>-0.2345142357877287</v>
       </c>
       <c r="S14" t="n">
-        <v>0.01186377529319393</v>
+        <v>0.1992889626887308</v>
       </c>
       <c r="T14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="U14" t="n">
-        <v>0.8516834718181404</v>
+        <v>0.8812693103954475</v>
       </c>
       <c r="V14" t="n">
-        <v>0.8450254130712601</v>
+        <v>0.9206776995403572</v>
       </c>
       <c r="W14" t="n">
-        <v>0.8483544424447003</v>
+        <v>0.9009735049679024</v>
       </c>
       <c r="X14" t="n">
-        <v>0.003329029373440151</v>
+        <v>0.01970419457245481</v>
       </c>
       <c r="Y14" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="Z14" t="n">
-        <v>0.06976286088804895</v>
+        <v>1.135487740755631</v>
       </c>
       <c r="AA14" t="n">
-        <v>0.7437101511126268</v>
+        <v>-0.8022581061655442</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.2240480184555054</v>
+        <v>0.384934663772583</v>
       </c>
       <c r="B15" t="n">
-        <v>0.05257594585418701</v>
+        <v>0.006433725357055664</v>
       </c>
       <c r="C15" t="n">
-        <v>0.08841598033905029</v>
+        <v>0.1532413959503174</v>
       </c>
       <c r="D15" t="n">
-        <v>0.02078831195831299</v>
+        <v>0.0002727508544921875</v>
       </c>
       <c r="E15" t="n">
-        <v>0.621999200099107</v>
+        <v>1.088923755064437</v>
       </c>
       <c r="F15" t="n">
-        <v>0.08792023670522557</v>
+        <v>0.0696604761871229</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -3386,83 +3504,83 @@
         <v>4</v>
       </c>
       <c r="I15" t="n">
-        <v>462</v>
+        <v>596</v>
       </c>
       <c r="J15" t="n">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="K15" t="n">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="L15" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="M15" t="n">
-        <v>5.908254330617086e-05</v>
+        <v>0.0002936060298520815</v>
       </c>
       <c r="N15" t="n">
-        <v>0.2273729743382297</v>
+        <v>0.202458944248629</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__l2_regularization': 0.621999200099107, 'model__learning_rate': 0.08792023670522557, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 462, 'model__max_leaf_nodes': 9, 'model__min_samples_leaf': 54, 'model__n_iter_no_change': 11, 'model__tol': 5.908254330617086e-05, 'model__validation_fraction': 0.22737297433822973})</t>
+          <t>OrderedDict({'model__l2_regularization': 1.0889237550644373, 'model__learning_rate': 0.0696604761871229, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 596, 'model__max_leaf_nodes': 22, 'model__min_samples_leaf': 59, 'model__n_iter_no_change': 18, 'model__tol': 0.00029360602985208155, 'model__validation_fraction': 0.20245894424862895})</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>0.7593522412062479</v>
+        <v>-0.08245734522395498</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.791870707530818</v>
+        <v>-0.4255670020290576</v>
       </c>
       <c r="R15" t="n">
-        <v>0.7756114743685329</v>
+        <v>-0.2540121736265063</v>
       </c>
       <c r="S15" t="n">
-        <v>0.01625923316228506</v>
+        <v>0.1715548284025513</v>
       </c>
       <c r="T15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="U15" t="n">
-        <v>0.8355224929576754</v>
+        <v>0.8985351703769541</v>
       </c>
       <c r="V15" t="n">
-        <v>0.8522085626477204</v>
+        <v>0.928640182774141</v>
       </c>
       <c r="W15" t="n">
-        <v>0.8438655278026979</v>
+        <v>0.9135876765755475</v>
       </c>
       <c r="X15" t="n">
-        <v>0.008343034845022468</v>
+        <v>0.01505250619859344</v>
       </c>
       <c r="Y15" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.06825405343416491</v>
+        <v>1.167599850202054</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.7414844476514505</v>
+        <v>-0.8378120987275331</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0.247681736946106</v>
+        <v>0.2843077182769775</v>
       </c>
       <c r="B16" t="n">
-        <v>0.001591324806213379</v>
+        <v>0.001500368118286133</v>
       </c>
       <c r="C16" t="n">
-        <v>0.09897458553314209</v>
+        <v>0.1130174398422241</v>
       </c>
       <c r="D16" t="n">
-        <v>0.0007461309432983398</v>
+        <v>0.002513289451599121</v>
       </c>
       <c r="E16" t="n">
-        <v>0.2940393582061399</v>
+        <v>0.621999200099107</v>
       </c>
       <c r="F16" t="n">
-        <v>0.08773835359169153</v>
+        <v>0.08792023670522557</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -3470,86 +3588,86 @@
         </is>
       </c>
       <c r="H16" t="n">
+        <v>4</v>
+      </c>
+      <c r="I16" t="n">
+        <v>462</v>
+      </c>
+      <c r="J16" t="n">
+        <v>9</v>
+      </c>
+      <c r="K16" t="n">
+        <v>54</v>
+      </c>
+      <c r="L16" t="n">
+        <v>11</v>
+      </c>
+      <c r="M16" t="n">
+        <v>5.908254330617086e-05</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0.2273729743382297</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>OrderedDict({'model__l2_regularization': 0.621999200099107, 'model__learning_rate': 0.08792023670522557, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 462, 'model__max_leaf_nodes': 9, 'model__min_samples_leaf': 54, 'model__n_iter_no_change': 11, 'model__tol': 5.908254330617086e-05, 'model__validation_fraction': 0.22737297433822973})</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>-0.06018201640402543</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>-0.4666333548700048</v>
+      </c>
+      <c r="R16" t="n">
+        <v>-0.2634076856370151</v>
+      </c>
+      <c r="S16" t="n">
+        <v>0.2032256692329897</v>
+      </c>
+      <c r="T16" t="n">
+        <v>15</v>
+      </c>
+      <c r="U16" t="n">
+        <v>0.8952060056633833</v>
+      </c>
+      <c r="V16" t="n">
+        <v>0.9232124366051632</v>
+      </c>
+      <c r="W16" t="n">
+        <v>0.9092092211342733</v>
+      </c>
+      <c r="X16" t="n">
+        <v>0.01400321547088995</v>
+      </c>
+      <c r="Y16" t="n">
         <v>3</v>
       </c>
-      <c r="I16" t="n">
-        <v>394</v>
-      </c>
-      <c r="J16" t="n">
-        <v>18</v>
-      </c>
-      <c r="K16" t="n">
-        <v>29</v>
-      </c>
-      <c r="L16" t="n">
-        <v>25</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0.000130220946023945</v>
-      </c>
-      <c r="N16" t="n">
-        <v>0.2465169071000755</v>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>OrderedDict({'model__l2_regularization': 0.2940393582061399, 'model__learning_rate': 0.08773835359169153, 'model__loss': 'squared_error', 'model__max_depth': 3, 'model__max_iter': 394, 'model__max_leaf_nodes': 18, 'model__min_samples_leaf': 29, 'model__n_iter_no_change': 25, 'model__tol': 0.000130220946023945, 'model__validation_fraction': 0.24651690710007554})</t>
-        </is>
-      </c>
-      <c r="P16" t="n">
-        <v>0.765257692130577</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>0.7838888421873917</v>
-      </c>
-      <c r="R16" t="n">
-        <v>0.7745732671589844</v>
-      </c>
-      <c r="S16" t="n">
-        <v>0.009315575028407352</v>
-      </c>
-      <c r="T16" t="n">
-        <v>14</v>
-      </c>
-      <c r="U16" t="n">
-        <v>0.8440287642696925</v>
-      </c>
-      <c r="V16" t="n">
-        <v>0.8388790310264036</v>
-      </c>
-      <c r="W16" t="n">
-        <v>0.8414538976480481</v>
-      </c>
-      <c r="X16" t="n">
-        <v>0.002574866621644467</v>
-      </c>
-      <c r="Y16" t="n">
-        <v>14</v>
-      </c>
       <c r="Z16" t="n">
-        <v>0.06688063048906367</v>
+        <v>1.172616906771288</v>
       </c>
       <c r="AA16" t="n">
-        <v>0.7411329519144526</v>
+        <v>-0.8497161390226593</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.3755068778991699</v>
+        <v>0.3309608697891235</v>
       </c>
       <c r="B17" t="n">
-        <v>0.01940631866455078</v>
+        <v>0.005258440971374512</v>
       </c>
       <c r="C17" t="n">
-        <v>0.1498433351516724</v>
+        <v>0.1281250715255737</v>
       </c>
       <c r="D17" t="n">
-        <v>0.008709311485290527</v>
+        <v>0.001944899559020996</v>
       </c>
       <c r="E17" t="n">
-        <v>4.358628897525027</v>
+        <v>0.2258215944659482</v>
       </c>
       <c r="F17" t="n">
-        <v>0.04047615571540435</v>
+        <v>0.0645191239031175</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -3560,83 +3678,83 @@
         <v>3</v>
       </c>
       <c r="I17" t="n">
-        <v>752</v>
+        <v>635</v>
       </c>
       <c r="J17" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="K17" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="L17" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="M17" t="n">
-        <v>5.083556924570688e-05</v>
+        <v>4.063746627400014e-05</v>
       </c>
       <c r="N17" t="n">
-        <v>0.2057254097308825</v>
+        <v>0.2042129064850941</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__l2_regularization': 4.358628897525027, 'model__learning_rate': 0.040476155715404354, 'model__loss': 'squared_error', 'model__max_depth': 3, 'model__max_iter': 752, 'model__max_leaf_nodes': 24, 'model__min_samples_leaf': 45, 'model__n_iter_no_change': 23, 'model__tol': 5.083556924570688e-05, 'model__validation_fraction': 0.20572540973088252})</t>
+          <t>OrderedDict({'model__l2_regularization': 0.22582159446594824, 'model__learning_rate': 0.0645191239031175, 'model__loss': 'squared_error', 'model__max_depth': 3, 'model__max_iter': 635, 'model__max_leaf_nodes': 18, 'model__min_samples_leaf': 41, 'model__n_iter_no_change': 25, 'model__tol': 4.063746627400014e-05, 'model__validation_fraction': 0.2042129064850941})</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>0.7495886504294695</v>
+        <v>-0.05733764602680047</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.7749659506562387</v>
+        <v>-0.4857119434107864</v>
       </c>
       <c r="R17" t="n">
-        <v>0.7622773005428541</v>
+        <v>-0.2715247947187934</v>
       </c>
       <c r="S17" t="n">
-        <v>0.0126886501133846</v>
+        <v>0.214187148691993</v>
       </c>
       <c r="T17" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="U17" t="n">
-        <v>0.8240365310493205</v>
+        <v>0.8793497537960676</v>
       </c>
       <c r="V17" t="n">
-        <v>0.8146180212497673</v>
+        <v>0.9179089268677679</v>
       </c>
       <c r="W17" t="n">
-        <v>0.8193272761495439</v>
+        <v>0.8986293403319178</v>
       </c>
       <c r="X17" t="n">
-        <v>0.004709254899776583</v>
+        <v>0.01927958653585016</v>
       </c>
       <c r="Y17" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="Z17" t="n">
-        <v>0.05704997560668978</v>
+        <v>1.170154135050711</v>
       </c>
       <c r="AA17" t="n">
-        <v>0.7337523127395092</v>
+        <v>-0.856601862244149</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0.2437286376953125</v>
+        <v>0.2029695510864258</v>
       </c>
       <c r="B18" t="n">
-        <v>0.01001167297363281</v>
+        <v>0.001455068588256836</v>
       </c>
       <c r="C18" t="n">
-        <v>0.09456014633178711</v>
+        <v>0.08202242851257324</v>
       </c>
       <c r="D18" t="n">
-        <v>0.003994464874267578</v>
+        <v>0.0004580020904541016</v>
       </c>
       <c r="E18" t="n">
-        <v>20</v>
+        <v>0.2940393582061399</v>
       </c>
       <c r="F18" t="n">
-        <v>0.1</v>
+        <v>0.08773835359169153</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -3647,83 +3765,83 @@
         <v>3</v>
       </c>
       <c r="I18" t="n">
-        <v>800</v>
+        <v>394</v>
       </c>
       <c r="J18" t="n">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="K18" t="n">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="L18" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="M18" t="n">
-        <v>0.001</v>
+        <v>0.000130220946023945</v>
       </c>
       <c r="N18" t="n">
-        <v>0.25</v>
+        <v>0.2465169071000755</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__l2_regularization': 20.0, 'model__learning_rate': 0.1, 'model__loss': 'squared_error', 'model__max_depth': 3, 'model__max_iter': 800, 'model__max_leaf_nodes': 31, 'model__min_samples_leaf': 80, 'model__n_iter_no_change': 10, 'model__tol': 0.001, 'model__validation_fraction': 0.25})</t>
+          <t>OrderedDict({'model__l2_regularization': 0.2940393582061399, 'model__learning_rate': 0.08773835359169153, 'model__loss': 'squared_error', 'model__max_depth': 3, 'model__max_iter': 394, 'model__max_leaf_nodes': 18, 'model__min_samples_leaf': 29, 'model__n_iter_no_change': 25, 'model__tol': 0.000130220946023945, 'model__validation_fraction': 0.24651690710007554})</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>0.7517757563944228</v>
+        <v>-0.04758097033997899</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.7744515723122958</v>
+        <v>-0.5098580331720635</v>
       </c>
       <c r="R18" t="n">
-        <v>0.7631136643533594</v>
+        <v>-0.2787195017560212</v>
       </c>
       <c r="S18" t="n">
-        <v>0.01133790795893647</v>
+        <v>0.2311385314160422</v>
       </c>
       <c r="T18" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="U18" t="n">
-        <v>0.823881796637664</v>
+        <v>0.8786451032931077</v>
       </c>
       <c r="V18" t="n">
-        <v>0.8217430185633748</v>
+        <v>0.9153710748342357</v>
       </c>
       <c r="W18" t="n">
-        <v>0.8228124076005194</v>
+        <v>0.8970080890636718</v>
       </c>
       <c r="X18" t="n">
-        <v>0.001069389037144597</v>
+        <v>0.018362985770564</v>
       </c>
       <c r="Y18" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="Z18" t="n">
-        <v>0.05969874324716007</v>
+        <v>1.175727590819693</v>
       </c>
       <c r="AA18" t="n">
-        <v>0.7332642927297793</v>
+        <v>-0.8665832971658677</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0.3948783874511719</v>
+        <v>0.2762755155563354</v>
       </c>
       <c r="B19" t="n">
-        <v>0.003502607345581055</v>
+        <v>0.00100100040435791</v>
       </c>
       <c r="C19" t="n">
-        <v>0.1569234132766724</v>
+        <v>0.1061645746231079</v>
       </c>
       <c r="D19" t="n">
-        <v>0.001865506172180176</v>
+        <v>0.0008312463760375977</v>
       </c>
       <c r="E19" t="n">
-        <v>4.80555470976749</v>
+        <v>14.25809463775946</v>
       </c>
       <c r="F19" t="n">
-        <v>0.02637321417594226</v>
+        <v>0.0617651314239038</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -3731,86 +3849,86 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I19" t="n">
-        <v>562</v>
+        <v>491</v>
       </c>
       <c r="J19" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="K19" t="n">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="L19" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="M19" t="n">
-        <v>0.0006665883558488896</v>
+        <v>0.0001544393009519414</v>
       </c>
       <c r="N19" t="n">
-        <v>0.1702833843482989</v>
+        <v>0.1428678327264134</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__l2_regularization': 4.80555470976749, 'model__learning_rate': 0.026373214175942256, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 562, 'model__max_leaf_nodes': 10, 'model__min_samples_leaf': 65, 'model__n_iter_no_change': 27, 'model__tol': 0.0006665883558488896, 'model__validation_fraction': 0.17028338434829887})</t>
+          <t>OrderedDict({'model__l2_regularization': 14.258094637759456, 'model__learning_rate': 0.0617651314239038, 'model__loss': 'squared_error', 'model__max_depth': 3, 'model__max_iter': 491, 'model__max_leaf_nodes': 13, 'model__min_samples_leaf': 20, 'model__n_iter_no_change': 17, 'model__tol': 0.00015443930095194143, 'model__validation_fraction': 0.1428678327264134})</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>0.7465959115449408</v>
+        <v>-0.06177094156622243</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.7644509821767878</v>
+        <v>-0.5024549066427928</v>
       </c>
       <c r="R19" t="n">
-        <v>0.7555234468608643</v>
+        <v>-0.2821129241045076</v>
       </c>
       <c r="S19" t="n">
-        <v>0.008927535315923496</v>
+        <v>0.2203419825382852</v>
       </c>
       <c r="T19" t="n">
         <v>18</v>
       </c>
       <c r="U19" t="n">
-        <v>0.8139250333272757</v>
+        <v>0.8766336044295446</v>
       </c>
       <c r="V19" t="n">
-        <v>0.7995115808035037</v>
+        <v>0.9096957179357896</v>
       </c>
       <c r="W19" t="n">
-        <v>0.8067183070653897</v>
+        <v>0.8931646611826671</v>
       </c>
       <c r="X19" t="n">
-        <v>0.00720672626188601</v>
+        <v>0.0165310567531225</v>
       </c>
       <c r="Y19" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="Z19" t="n">
-        <v>0.05119486020452546</v>
+        <v>1.175277585287175</v>
       </c>
       <c r="AA19" t="n">
-        <v>0.7299260167586015</v>
+        <v>-0.8697517167480949</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0.2796951532363892</v>
+        <v>0.3610688447952271</v>
       </c>
       <c r="B20" t="n">
-        <v>0.006157517433166504</v>
+        <v>0.09141123294830322</v>
       </c>
       <c r="C20" t="n">
-        <v>0.1209871768951416</v>
+        <v>0.133453369140625</v>
       </c>
       <c r="D20" t="n">
-        <v>0.002829790115356445</v>
+        <v>0.03297567367553711</v>
       </c>
       <c r="E20" t="n">
-        <v>2.648795958041073</v>
+        <v>5.810909071553644</v>
       </c>
       <c r="F20" t="n">
-        <v>0.09070291931029359</v>
+        <v>0.08287830852695076</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -3818,86 +3936,86 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I20" t="n">
-        <v>700</v>
+        <v>732</v>
       </c>
       <c r="J20" t="n">
+        <v>9</v>
+      </c>
+      <c r="K20" t="n">
+        <v>28</v>
+      </c>
+      <c r="L20" t="n">
         <v>17</v>
       </c>
-      <c r="K20" t="n">
-        <v>48</v>
-      </c>
-      <c r="L20" t="n">
-        <v>21</v>
-      </c>
       <c r="M20" t="n">
-        <v>0.0003720213584666978</v>
+        <v>0.0001868349859728154</v>
       </c>
       <c r="N20" t="n">
-        <v>0.192465536472899</v>
+        <v>0.2439524195246732</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__l2_regularization': 2.648795958041073, 'model__learning_rate': 0.09070291931029359, 'model__loss': 'squared_error', 'model__max_depth': 2, 'model__max_iter': 700, 'model__max_leaf_nodes': 17, 'model__min_samples_leaf': 48, 'model__n_iter_no_change': 21, 'model__tol': 0.0003720213584666978, 'model__validation_fraction': 0.19246553647289905})</t>
+          <t>OrderedDict({'model__l2_regularization': 5.8109090715536444, 'model__learning_rate': 0.08287830852695076, 'model__loss': 'squared_error', 'model__max_depth': 4, 'model__max_iter': 732, 'model__max_leaf_nodes': 9, 'model__min_samples_leaf': 28, 'model__n_iter_no_change': 17, 'model__tol': 0.00018683498597281536, 'model__validation_fraction': 0.24395241952467317})</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>0.7316785747686914</v>
+        <v>-0.0642859632151751</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.7542616952837419</v>
+        <v>-0.5273924310880267</v>
       </c>
       <c r="R20" t="n">
-        <v>0.7429701350262166</v>
+        <v>-0.2958391971516009</v>
       </c>
       <c r="S20" t="n">
-        <v>0.01129156025752526</v>
+        <v>0.2315532339364258</v>
       </c>
       <c r="T20" t="n">
         <v>19</v>
       </c>
       <c r="U20" t="n">
-        <v>0.8018327032421055</v>
+        <v>0.9174784865572941</v>
       </c>
       <c r="V20" t="n">
-        <v>0.7921489477251756</v>
+        <v>0.9287838490387268</v>
       </c>
       <c r="W20" t="n">
-        <v>0.7969908254836406</v>
+        <v>0.9231311677980105</v>
       </c>
       <c r="X20" t="n">
-        <v>0.004841877758464952</v>
+        <v>0.005652681240716328</v>
       </c>
       <c r="Y20" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="Z20" t="n">
-        <v>0.05402069045742408</v>
+        <v>1.218970364949612</v>
       </c>
       <c r="AA20" t="n">
-        <v>0.7159597897975045</v>
+        <v>-0.9053243796264067</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.144291877746582</v>
+        <v>0.2983976602554321</v>
       </c>
       <c r="B21" t="n">
-        <v>0.0008740425109863281</v>
+        <v>5.960464477539062e-07</v>
       </c>
       <c r="C21" t="n">
-        <v>0.05354893207550049</v>
+        <v>0.1150722503662109</v>
       </c>
       <c r="D21" t="n">
-        <v>0.000630497932434082</v>
+        <v>2.384185791015625e-07</v>
       </c>
       <c r="E21" t="n">
-        <v>3.095552171571063</v>
+        <v>2.648795958041073</v>
       </c>
       <c r="F21" t="n">
-        <v>0.02</v>
+        <v>0.09070291931029359</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -3908,63 +4026,63 @@
         <v>2</v>
       </c>
       <c r="I21" t="n">
-        <v>300</v>
+        <v>700</v>
       </c>
       <c r="J21" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="K21" t="n">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="L21" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="M21" t="n">
-        <v>1.121142034442108e-05</v>
+        <v>0.0003720213584666978</v>
       </c>
       <c r="N21" t="n">
-        <v>0.1558402881414565</v>
+        <v>0.192465536472899</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>OrderedDict({'model__l2_regularization': 3.0955521715710628, 'model__learning_rate': 0.020000000000000004, 'model__loss': 'squared_error', 'model__max_depth': 2, 'model__max_iter': 300, 'model__max_leaf_nodes': 27, 'model__min_samples_leaf': 31, 'model__n_iter_no_change': 16, 'model__tol': 1.121142034442108e-05, 'model__validation_fraction': 0.15584028814145645})</t>
+          <t>OrderedDict({'model__l2_regularization': 2.648795958041073, 'model__learning_rate': 0.09070291931029359, 'model__loss': 'squared_error', 'model__max_depth': 2, 'model__max_iter': 700, 'model__max_leaf_nodes': 17, 'model__min_samples_leaf': 48, 'model__n_iter_no_change': 21, 'model__tol': 0.0003720213584666978, 'model__validation_fraction': 0.19246553647289905})</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>0.6076607009568342</v>
+        <v>-0.07508915078881362</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.6532931326072005</v>
+        <v>-0.5552478052181689</v>
       </c>
       <c r="R21" t="n">
-        <v>0.6304769167820173</v>
+        <v>-0.3151684780034912</v>
       </c>
       <c r="S21" t="n">
-        <v>0.02281621582518312</v>
+        <v>0.2400793272146776</v>
       </c>
       <c r="T21" t="n">
         <v>20</v>
       </c>
       <c r="U21" t="n">
-        <v>0.6579589086520669</v>
+        <v>0.8524182402253164</v>
       </c>
       <c r="V21" t="n">
-        <v>0.6432317298167463</v>
+        <v>0.890915099648848</v>
       </c>
       <c r="W21" t="n">
-        <v>0.6505953192344065</v>
+        <v>0.8716666699370822</v>
       </c>
       <c r="X21" t="n">
-        <v>0.007363589417660299</v>
+        <v>0.01924842971176577</v>
       </c>
       <c r="Y21" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="Z21" t="n">
-        <v>0.02011840245238916</v>
+        <v>1.186835147940573</v>
       </c>
       <c r="AA21" t="n">
-        <v>0.6204177155558228</v>
+        <v>-0.908586051973778</v>
       </c>
     </row>
   </sheetData>
@@ -4001,53 +4119,53 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>bitsize</t>
+          <t>mw_in</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.3978110445573936</v>
+        <v>0.2136835530050681</v>
       </c>
       <c r="C2" t="n">
-        <v>0.01028628652656488</v>
+        <v>0.008052468123663633</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>mw_in</t>
+          <t>bitsize</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.3554501653325289</v>
+        <v>0.2003954358662979</v>
       </c>
       <c r="C3" t="n">
-        <v>0.008932025297177015</v>
+        <v>0.007790050656415504</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>torque</t>
+          <t>flowrate</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1938354284961027</v>
+        <v>0.1048214540004793</v>
       </c>
       <c r="C4" t="n">
-        <v>0.008236637319160099</v>
+        <v>0.005885167850236321</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>flowrate</t>
+          <t>torque</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.1645239920978383</v>
+        <v>0.07842470500013166</v>
       </c>
       <c r="C5" t="n">
-        <v>0.003090030661934848</v>
+        <v>0.004993909211996759</v>
       </c>
     </row>
     <row r="6">
@@ -4057,10 +4175,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.1023731793899852</v>
+        <v>0.02486850034807715</v>
       </c>
       <c r="C6" t="n">
-        <v>0.005164505450284649</v>
+        <v>0.001422801412419581</v>
       </c>
     </row>
     <row r="7">
@@ -4070,10 +4188,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.09897674874736563</v>
+        <v>0.02194535126396992</v>
       </c>
       <c r="C7" t="n">
-        <v>0.003234024561039688</v>
+        <v>0.003697615325010382</v>
       </c>
     </row>
     <row r="8">
@@ -4083,10 +4201,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.08879283210068196</v>
+        <v>0.02081024129989046</v>
       </c>
       <c r="C8" t="n">
-        <v>0.001804210753916976</v>
+        <v>0.002376061169511858</v>
       </c>
     </row>
   </sheetData>

</xml_diff>